<commit_message>
docs: corrige o numero da coluna do portal (tela tem filtro de periodo)
A tela do Onboarding tem filtro de periodo: o 202 era "Ultimos 30 dias".
Com "Todo o periodo" a coluna Formulario do varejo pendente mostra 446.
A API devolve 473 em dados_varejo, e os 27 de diferenca sao exatamente os
que tem unblinded_at preenchido - unico campo que separa 473 em 446+27.

O resto da conferencia nao muda: 403 cards distintos por tras desses CNPJs
contra 334 na etapa 50 do Evo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Etapa50-x-dados_varejo-2026-10-19.xlsx
+++ b/docs/Etapa50-x-dados_varejo-2026-10-19.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr"/>
@@ -505,336 +506,381 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>A tela do portal mostra só os últimos 30 dias</t>
+          <t>Tela com "Todo o período"</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>202</v>
+        <v>446</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>é o "202": onboardings em dados_varejo criados nos últimos 30 dias</t>
+          <t>o que o portal mostra na coluna quando o filtro de período é removido (Aldo, 19/10)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Em dados_varejo há mais de 30 dias</t>
+          <t>API em dados_varejo</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>271</v>
+        <v>473</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>existem no portal, não aparecem naquela tela</t>
+          <t>27 a mais que a tela: são exatamente os 27 com unblinded_at preenchido</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Total real em dados_varejo (CNPJs)</t>
+          <t>Diferença tela x API</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>473</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>202 + 271 — o portal tem MAIS pendente do que mostra</t>
+          <t>único campo que separa 473 em 446+27 — confirmar com o Mauricio o que a tela faz com eles</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cards distintos por trás desses CNPJs</t>
+          <t>A tela do portal mostra só os últimos 30 dias</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>403</v>
+        <v>202</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>matriz e filiais somam CNPJ, mas são um card só</t>
+          <t>é o "202" que você viu: o filtro de período estava em 30 dias</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Cards na etapa 50 do Evo</t>
+          <t>Em dados_varejo há mais de 30 dias</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>334</v>
+        <v>271</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>o "300 e poucos"</t>
+          <t>existem no portal, não aparecem naquela tela</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Total real em dados_varejo (CNPJs)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>473</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>202 + 271 — o portal tem MAIS pendente do que mostra</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>PORTAL DA AIVA (Track) — 859 onboardings</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr"/>
+          <t>Cards distintos por trás desses CNPJs</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>403</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>matriz e filiais somam CNPJ, mas são um card só</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  coluna dados_varejo</t>
+          <t>Cards na etapa 50 do Evo</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>473</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr"/>
+        <v>334</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>o "300 e poucos"</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  coluna not_approved</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>27</v>
-      </c>
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  coluna cadastro_finalizado</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>322</v>
-      </c>
+          <t>PORTAL DA AIVA (Track) — 859 onboardings</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  coluna biometria</t>
+          <t xml:space="preserve">  coluna dados_varejo</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>36</v>
+        <v>473</v>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  coluna pre_cadastro</t>
+          <t xml:space="preserve">  coluna not_approved</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  coluna cadastro_finalizado</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>322</v>
+      </c>
       <c r="C18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>EVO — funil 15 por etapa</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
+          <t xml:space="preserve">  coluna biometria</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>36</v>
+      </c>
       <c r="C19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 66</t>
+          <t xml:space="preserve">  coluna pre_cadastro</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>9723</v>
+        <v>1</v>
       </c>
       <c r="C20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  etapa 53</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>6119</v>
-      </c>
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 47</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>2457</v>
-      </c>
+          <t>EVO — funil 15 por etapa</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 50</t>
+          <t xml:space="preserve">  etapa 66</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>334</v>
+        <v>9723</v>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 51</t>
+          <t xml:space="preserve">  etapa 53</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>254</v>
+        <v>6119</v>
       </c>
       <c r="C24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 69</t>
+          <t xml:space="preserve">  etapa 47</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>211</v>
+        <v>2457</v>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 71</t>
+          <t xml:space="preserve">  etapa 50</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>49</v>
+        <v>334</v>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 93</t>
+          <t xml:space="preserve">  etapa 51</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>47</v>
+        <v>254</v>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 94</t>
+          <t xml:space="preserve">  etapa 69</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>24</v>
+        <v>211</v>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 99</t>
+          <t xml:space="preserve">  etapa 71</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 95</t>
+          <t xml:space="preserve">  etapa 93</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="C30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 96</t>
+          <t xml:space="preserve">  etapa 94</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 70</t>
+          <t xml:space="preserve">  etapa 99</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 49</t>
+          <t xml:space="preserve">  etapa 95</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  etapa 54</t>
+          <t xml:space="preserve">  etapa 96</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  etapa 70</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  etapa 49</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  etapa 54</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  etapa 97</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n">
+      <c r="B38" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>